<commit_message>
hot rolled resu mod variable
</commit_message>
<xml_diff>
--- a/parameters_section_HEB.xlsx
+++ b/parameters_section_HEB.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="116" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="124" uniqueCount="4">
   <si>
     <t>i</t>
   </si>
@@ -418,10 +418,10 @@
   <dimension ref="A1:G97"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="true"/>
-    <col min="2" max="2" width="2.42578125" customWidth="true"/>
-    <col min="4" max="4" width="3.42578125" customWidth="true"/>
-    <col min="3" max="3" width="3.7109375" customWidth="true"/>
+    <col min="1" max="1" width="1.3203125" customWidth="true"/>
+    <col min="2" max="2" width="2.08984375" customWidth="true"/>
+    <col min="4" max="4" width="3.08984375" customWidth="true"/>
+    <col min="3" max="3" width="3.26953125" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.25">

</xml_diff>